<commit_message>
chore(eval): 골든셋 cycle 교정 + PLAN-019 작업 로그 정리
골든셋 수정 (v1_1 잔존 실패 분석 후):
- conf_007 ICMF: cycle_years 2→3, upcoming_start/end 공란화 (미공개 수용)
- conf_017 PRTEC: cycle_years 4→3

PLAN-019.md:
- Step 1~10 전부 체크 (v1_0 작성 → 측정 → v1_1 작성 → 측정 → 잔존 분석)
- §8 후속 항목 재정비 — conf_006 date null·conf_007 JSON 안정성·conf_017 DB cycle 교정·BS2027 실질적 성공 판단
- §9 작업 로그 하루 흐름 상세 기록 (f928faa → d1a549d → 861e799)

주의: public/data/conferences.json 의 cycle_years 는 미수정.
프롬프트 input 교정은 다음 세션 v1_2 에서 묶어서 진행 예정.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/eval/golden-set.xlsx
+++ b/docs/eval/golden-set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerom\ConferenceFinder\docs\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF0045FB-F638-4026-BFDE-7740EB6AE98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857218AD-37DD-476C-BCD9-4D756CEA72A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="golden" sheetId="1" r:id="rId1"/>
@@ -2018,7 +2018,7 @@
         <v>87</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8">
         <v>5</v>
@@ -2756,7 +2756,7 @@
         <v>87</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18">
         <v>4</v>
@@ -3587,7 +3587,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:X1 A28:B28 A10:N10 A2:I2 K2:T2 A3:I3 K3:N3 A4:I4 K4:N4 A5:I5 K5:X5 A6:I6 K6 A7:I7 K7:N7 A8:B8 D8:M8 A9:B9 D9:N9 A13:I13 A11:I11 K11:X11 A12:I12 K12:O12 A16:I16 A14:B14 D14:I14 K14:X14 K13:N13 A15:I15 K15:X15 A18:X19 A17:I17 K17:X17 A23:N23 A21:I21 K21:N21 A22 C22:I22 K22:N22 A25:N25 A24:I24 K24:N24 A27:B27 A26:B26 K26:N26 D28:O28 D26:G26 I26 D27:G27 I27:N27 Q4:X4 Q8:X8 Q12:X12 P16:T16 A20:N20 Q20:X20 P21:X21 P22:X22 P23:X23 P24:T24 P25:X25 P26:T26 P27:T27 Q28:X28 V2:X2 V3:X3 P3:T3 V6:X6 P6:T6 V7:X7 V9:X9 P9:T9 V10:X10 V24:X24 V26:X26 P13:T13 P10:T10 P7:T7 K16:N16 V16:X16 V13:X13 V27:X27" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:X1 A28:B28 A10:N10 A2:I2 K2:T2 A3:I3 K3:N3 A4:I4 K4:N4 A5:I5 K5:X5 A6:I6 K6 A7:I7 K7:N7 A8:B8 D8:F8 A9:B9 D9:N9 A13:I13 A11:I11 K11:X11 A12:I12 K12:O12 A16:I16 A14:B14 D14:I14 K14:X14 K13:N13 A15:I15 K15:X15 A19:X19 A17:I17 K17:X17 A23:N23 A21:I21 K21:N21 A22 C22:I22 K22:N22 A25:N25 A24:I24 K24:N24 A27:B27 A26:B26 K26:N26 D28:O28 D26:G26 I26 D27:G27 I27:N27 Q4:X4 Q8:X8 Q12:X12 P16:T16 A20:N20 Q20:X20 P21:X21 P22:X22 P23:X23 P24:T24 P25:X25 P26:T26 P27:T27 Q28:X28 V2:X2 V3:X3 P3:T3 V6:X6 P6:T6 V7:X7 V9:X9 P9:T9 V10:X10 V24:X24 V26:X26 P13:T13 P10:T10 P7:T7 K16:N16 V16:X16 V13:X13 V27:X27 H8:M8 A18:F18 H18:X18" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>